<commit_message>
data: finalize XSMB 2026-08-31
</commit_message>
<xml_diff>
--- a/data/excel/xsmb-2-digits.xlsx
+++ b/data/excel/xsmb-2-digits.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TwoDigits" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$386</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$387</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB386"/>
+  <dimension ref="A1:AB387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55275,8 +55275,150 @@
         </is>
       </c>
     </row>
+    <row r="387">
+      <c r="A387" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B387" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="C387" s="2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="D387" s="2" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="E387" s="2" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="F387" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="G387" s="2" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="H387" s="2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="I387" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="J387" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="K387" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="L387" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="M387" s="2" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="N387" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="O387" s="2" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="P387" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="Q387" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="R387" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="S387" s="2" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="T387" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="U387" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="V387" s="2" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="W387" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="X387" s="2" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="Y387" s="2" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="Z387" s="2" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="AA387" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="AB387" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB386"/>
+  <autoFilter ref="A1:AB387"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: finalize XSMB 2026-09-01
</commit_message>
<xml_diff>
--- a/data/excel/xsmb-2-digits.xlsx
+++ b/data/excel/xsmb-2-digits.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TwoDigits" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$387</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$388</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB387"/>
+  <dimension ref="A1:AB388"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55417,8 +55417,150 @@
         </is>
       </c>
     </row>
+    <row r="388">
+      <c r="A388" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B388" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C388" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="D388" s="2" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="E388" s="2" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="F388" s="2" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
+      <c r="G388" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="H388" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="I388" s="2" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="J388" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="K388" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="L388" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="M388" s="2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="N388" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="O388" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="P388" s="2" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="Q388" s="2" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="R388" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="S388" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="T388" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="U388" s="2" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="V388" s="2" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="W388" s="2" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="X388" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="Y388" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="Z388" s="2" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="AA388" s="2" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="AB388" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB387"/>
+  <autoFilter ref="A1:AB388"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: finalize XSMB 2026-09-02
</commit_message>
<xml_diff>
--- a/data/excel/xsmb-2-digits.xlsx
+++ b/data/excel/xsmb-2-digits.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TwoDigits" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$388</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$389</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB388"/>
+  <dimension ref="A1:AB389"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55559,8 +55559,150 @@
         </is>
       </c>
     </row>
+    <row r="389">
+      <c r="A389" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B389" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="C389" s="2" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="D389" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="E389" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="F389" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="G389" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="H389" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I389" s="2" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="J389" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="K389" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="L389" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="M389" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="N389" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="O389" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="P389" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="Q389" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="R389" s="2" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="S389" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="T389" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="U389" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="V389" s="2" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="W389" s="2" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="X389" s="2" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="Y389" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="Z389" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="AA389" s="2" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="AB389" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB388"/>
+  <autoFilter ref="A1:AB389"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: finalize XSMB 2026-09-03
</commit_message>
<xml_diff>
--- a/data/excel/xsmb-2-digits.xlsx
+++ b/data/excel/xsmb-2-digits.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TwoDigits" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$389</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$390</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB389"/>
+  <dimension ref="A1:AB390"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55701,8 +55701,150 @@
         </is>
       </c>
     </row>
+    <row r="390">
+      <c r="A390" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B390" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C390" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="D390" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E390" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="F390" s="2" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="G390" s="2" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="H390" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="I390" s="2" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="J390" s="2" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="K390" s="2" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="L390" s="2" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="M390" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="N390" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="O390" s="2" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="P390" s="2" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="Q390" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="R390" s="2" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="S390" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T390" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="U390" s="2" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="V390" s="2" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
+      <c r="W390" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="X390" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="Y390" s="2" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z390" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="AA390" s="2" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="AB390" s="2" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB389"/>
+  <autoFilter ref="A1:AB390"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: finalize XSMB 2026-09-04
</commit_message>
<xml_diff>
--- a/data/excel/xsmb-2-digits.xlsx
+++ b/data/excel/xsmb-2-digits.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TwoDigits" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$390</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$391</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB390"/>
+  <dimension ref="A1:AB391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55843,8 +55843,150 @@
         </is>
       </c>
     </row>
+    <row r="391">
+      <c r="A391" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B391" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="C391" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="D391" s="2" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="E391" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="F391" s="2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="G391" s="2" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="H391" s="2" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+      <c r="I391" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="J391" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="K391" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="L391" s="2" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="M391" s="2" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="N391" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="O391" s="2" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="P391" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="Q391" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="R391" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="S391" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="T391" s="2" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="U391" s="2" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="V391" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="W391" s="2" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="X391" s="2" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="Y391" s="2" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="Z391" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="AA391" s="2" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="AB391" s="2" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB390"/>
+  <autoFilter ref="A1:AB391"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: finalize XSMB 2026-09-05
</commit_message>
<xml_diff>
--- a/data/excel/xsmb-2-digits.xlsx
+++ b/data/excel/xsmb-2-digits.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TwoDigits" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$391</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$392</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB391"/>
+  <dimension ref="A1:AB392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55985,8 +55985,150 @@
         </is>
       </c>
     </row>
+    <row r="392">
+      <c r="A392" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B392" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="C392" s="2" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="D392" s="2" t="inlineStr">
+        <is>
+          <t>94</t>
+        </is>
+      </c>
+      <c r="E392" s="2" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="F392" s="2" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="G392" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="H392" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="I392" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J392" s="2" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="K392" s="2" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="L392" s="2" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
+      <c r="M392" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="N392" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="O392" s="2" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="P392" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="Q392" s="2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="R392" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="S392" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="T392" s="2" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="U392" s="2" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="V392" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="W392" s="2" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="X392" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="Y392" s="2" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="Z392" s="2" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="AA392" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="AB392" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB391"/>
+  <autoFilter ref="A1:AB392"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: finalize XSMB 2026-09-06
</commit_message>
<xml_diff>
--- a/data/excel/xsmb-2-digits.xlsx
+++ b/data/excel/xsmb-2-digits.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TwoDigits" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$392</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$393</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB392"/>
+  <dimension ref="A1:AB393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -56127,8 +56127,150 @@
         </is>
       </c>
     </row>
+    <row r="393">
+      <c r="A393" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B393" s="2" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="C393" s="2" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="D393" s="2" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="E393" s="2" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="F393" s="2" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="G393" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="H393" s="2" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="I393" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="J393" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="K393" s="2" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="L393" s="2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="M393" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="N393" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="O393" s="2" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="P393" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="Q393" s="2" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="R393" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="S393" s="2" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="T393" s="2" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+      <c r="U393" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="V393" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="W393" s="2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="X393" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="Y393" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="Z393" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="AA393" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="AB393" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB392"/>
+  <autoFilter ref="A1:AB393"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: finalize XSMB 2026-09-07
</commit_message>
<xml_diff>
--- a/data/excel/xsmb-2-digits.xlsx
+++ b/data/excel/xsmb-2-digits.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TwoDigits" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$393</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TwoDigits'!$A$1:$AB$394</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB393"/>
+  <dimension ref="A1:AB394"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -56269,8 +56269,150 @@
         </is>
       </c>
     </row>
+    <row r="394">
+      <c r="A394" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B394" s="2" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="C394" s="2" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="D394" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="E394" s="2" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="F394" s="2" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="G394" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="H394" s="2" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="I394" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="J394" s="2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="K394" s="2" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="L394" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="M394" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="N394" s="2" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="O394" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="P394" s="2" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="Q394" s="2" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="R394" s="2" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="S394" s="2" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="T394" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="U394" s="2" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="V394" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="W394" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="X394" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="Y394" s="2" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="Z394" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="AA394" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB394" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB393"/>
+  <autoFilter ref="A1:AB394"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>